<commit_message>
Ship verified APC40 visual twin release
</commit_message>
<xml_diff>
--- a/docs/APC40_Visual_QA_Control_Map.xlsx
+++ b/docs/APC40_Visual_QA_Control_Map.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R25e64b1213ca4195"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Map" sheetId="2" r:id="Re881f9e2777d45c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="XML Shortcuts" sheetId="3" r:id="Re19fb7d2e5464b5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuous Detail" sheetId="4" r:id="R96ef6e3052354014"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Button Feedback" sheetId="5" r:id="Rfdade5b68bdc444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Checks" sheetId="6" r:id="R18ddd90e7e124018"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rbd343518d13241c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Map" sheetId="2" r:id="R64b53ca9abe149ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="XML Shortcuts" sheetId="3" r:id="R8dc83005766a4bae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Continuous Detail" sheetId="4" r:id="Rd5df42b4a269429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Button Feedback" sheetId="5" r:id="R5be4ae1fa55949dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Checks" sheetId="6" r:id="R3524973212d943b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -334,7 +334,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -345,7 +345,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -356,7 +356,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -367,7 +367,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -378,7 +378,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -389,7 +389,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -400,7 +400,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -411,7 +411,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -422,7 +422,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -433,7 +433,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -444,7 +444,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -455,7 +455,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -1006,7 +1006,7 @@
         <x:v>Source XML</x:v>
       </x:c>
       <x:c r="B10" s="31" t="str">
-        <x:v>C:/Users/jeffr/OneDrive/Documents/Resolume Avenue/Shortcuts/MIDI/APC 40 MK II - Visual QA.xml</x:v>
+        <x:v>controllers/APC 40 MK II - Visual QA.xml</x:v>
       </x:c>
       <x:c r="C10" s="31"/>
       <x:c r="D10" s="31" t="str">
@@ -1197,7 +1197,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5b565cbf9e34483"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b5195ed94de401c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10602,7 +10602,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R108a657e652e4704"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0299a6382be74b00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24388,7 +24388,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14b9f308fb2646db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3456a05b132c42ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26061,7 +26061,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R956d0cadb712451c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63cae93556984aeb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31510,7 +31510,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdea4bae3b35b4618"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d4b2e3c25b945ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31892,7 +31892,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ea66457d31940df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde4b7a29ae934979"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>